<commit_message>
docs(QA): calificar HU-17 como EN REVISION por pendiente en Google Sheets (CA4)
</commit_message>
<xml_diff>
--- a/Docs/Matriz_QA_Aprobacion_Oficial.xlsx
+++ b/Docs/Matriz_QA_Aprobacion_Oficial.xlsx
@@ -768,10 +768,14 @@
       </c>
       <c r="H8" s="10" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="I8" s="10" t="inlineStr"/>
+          <t>EN REVISIÓN</t>
+        </is>
+      </c>
+      <c r="I8" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
       <c r="J8" s="9" t="inlineStr">
         <is>
           <t>CA1. Se presenta el radar del filtro de idoneidad.
@@ -782,7 +786,7 @@
       </c>
       <c r="K8" s="9" t="inlineStr">
         <is>
-          <t>Devolver al responsable para subsanar los criterios no cumplidos</t>
+          <t>EN REVISIÓN: Análisis conceptual y radar de idoneidad excelentes (cumple CA1, CA2 y CA3). Pendiente cargar información en la hoja PROYECTO de Google Sheets (CA4).</t>
         </is>
       </c>
     </row>

</xml_diff>